<commit_message>
Add comments and docstrings to code. Add README files to folders. Make codebase neater.
</commit_message>
<xml_diff>
--- a/results_single/results_single.xlsx
+++ b/results_single/results_single.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leticiadupleich/Desktop/Capstone/LeticiaCapstone/results_single/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AE5B40E-B3B3-E54C-991D-1AFD91D5A8C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69870E73-5E87-D347-8E8E-04BB3CB0AF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16300" activeTab="3" xr2:uid="{F1D71396-1DC3-294D-A1BC-F6200886B423}"/>
   </bookViews>
@@ -98,9 +98,6 @@
     <t>elapsed_ms</t>
   </si>
   <si>
-    <t>Elapsed Time</t>
-  </si>
-  <si>
     <t>CPU Time</t>
   </si>
   <si>
@@ -126,6 +123,9 @@
   </si>
   <si>
     <t>Single Elapsed Time SQL</t>
+  </si>
+  <si>
+    <t>Execution Time</t>
   </si>
 </sst>
 </file>
@@ -1550,7 +1550,7 @@
                   <a:schemeClr val="tx1"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Comparison of Elapsed Time and CPU Time for </a:t>
+              <a:t>Comparison of Execution Time and CPU Time for </a:t>
             </a:r>
             <a:r>
               <a:rPr lang="en-GB" sz="1400" b="1" i="1" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
@@ -1615,7 +1615,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Elapsed Time</c:v>
+                  <c:v>Execution Time</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5991,7 +5991,7 @@
                   <a:schemeClr val="tx1"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Comparison of Elapsed Time and</a:t>
+              <a:t>Comparison of Execution Time and</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="en-GB" b="1" baseline="0">
@@ -6084,7 +6084,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Elapsed Time</c:v>
+                  <c:v>Execution Time</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -7109,7 +7109,7 @@
                   <a:schemeClr val="tx1"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Comparison of Elapsed Time and CPU Time for </a:t>
+              <a:t>Comparison of Execution Time and CPU Time for </a:t>
             </a:r>
             <a:r>
               <a:rPr lang="en-GB" sz="1400" b="1" i="1" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
@@ -7174,7 +7174,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Elapsed Time</c:v>
+                  <c:v>Execution Time</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -8190,7 +8190,7 @@
                   <a:schemeClr val="tx1"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Comparison of Elapsed Time and CPU Time for </a:t>
+              <a:t>Comparison of Execution Time and CPU Time for </a:t>
             </a:r>
             <a:r>
               <a:rPr lang="en-GB" sz="1400" b="1" i="1" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
@@ -8255,7 +8255,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Elapsed Time</c:v>
+                  <c:v>Execution Time</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -15469,7 +15469,7 @@
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
       <c r="E1" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -15537,7 +15537,7 @@
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
       <c r="E8" s="22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F8" s="23"/>
       <c r="G8" s="24"/>
@@ -17889,7 +17889,7 @@
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
       <c r="E1" s="27" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F1" s="27"/>
       <c r="G1" s="27"/>
@@ -17957,7 +17957,7 @@
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
       <c r="E8" s="27" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F8" s="27"/>
       <c r="G8" s="27"/>
@@ -18046,7 +18046,7 @@
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
       <c r="E1" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -18114,7 +18114,7 @@
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
       <c r="E8" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
@@ -18197,48 +18197,48 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="7"/>
       <c r="D1" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E1" s="8"/>
       <c r="G1" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H1" s="8"/>
       <c r="J1" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="K1" s="8"/>
     </row>
     <row r="2" spans="1:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>18</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>19</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="11" t="s">
-        <v>19</v>
-      </c>
       <c r="G2" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="11" t="s">
-        <v>19</v>
-      </c>
       <c r="J2" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="K2" s="11" t="s">
         <v>18</v>
-      </c>
-      <c r="K2" s="11" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -21483,7 +21483,7 @@
         <v>0.44608116149902299</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
@@ -28268,7 +28268,7 @@
         <v>0.27799606323242099</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>

</xml_diff>